<commit_message>
Make treatment label name a setting in the Excel metadata
</commit_message>
<xml_diff>
--- a/data-raw/metadata.xlsx
+++ b/data-raw/metadata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lsamson\Projects\99 - Statistial and data projects\IMpress\clinsight\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96A7620C-32CD-4537-B780-487F008F2C10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAA231DE-F3AC-4A79-955E-2D8F4020D518}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{3E8FFA66-BACE-4C4A-A255-562C367A8A13}"/>
+    <workbookView xWindow="28680" yWindow="0" windowWidth="21600" windowHeight="11295" activeTab="7" xr2:uid="{3E8FFA66-BACE-4C4A-A255-562C367A8A13}"/>
   </bookViews>
   <sheets>
     <sheet name="column_names" sheetId="17" r:id="rId1"/>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="538" uniqueCount="298">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="540" uniqueCount="300">
   <si>
     <t>continuous</t>
   </si>
@@ -968,6 +968,12 @@
   </si>
   <si>
     <t>expected_events</t>
+  </si>
+  <si>
+    <t>treatment_label</t>
+  </si>
+  <si>
+    <t>\U1F48A T\U2093</t>
   </si>
 </sst>
 </file>
@@ -3601,16 +3607,16 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D2F7ED2-3887-47C4-B9C3-26B3456EF3BF}">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="30" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="25.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="24" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="25.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>277</v>
       </c>
@@ -3623,8 +3629,11 @@
       <c r="D1" t="s">
         <v>276</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>278</v>
       </c>
@@ -3633,6 +3642,9 @@
       </c>
       <c r="D2" t="s">
         <v>275</v>
+      </c>
+      <c r="E2" t="s">
+        <v>299</v>
       </c>
     </row>
   </sheetData>

</xml_diff>